<commit_message>
vault backup: 2026-07-14 17:25:28
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/软件概要设计-模块功能拆分-v2.xlsx
+++ b/公司项目/认知作战/文档/软件概要设计-模块功能拆分-v2.xlsx
@@ -8139,11 +8139,11 @@
       <x:c r="C2" s="3" t="s">
         <x:v>713</x:v>
       </x:c>
-      <x:c r="D2" s="3" t="s">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="E2" s="3" t="s">
-        <x:v>126</x:v>
+      <x:c r="D2" s="3" t="str">
+        <x:v>R-SWM-001~005</x:v>
+      </x:c>
+      <x:c r="E2" s="3" t="str">
+        <x:v>执行层的「提示词生成与记忆中心」：根据人设(画像/账号属性)生成驱动智能体作业的提示词并管理记忆，将生成的提示词包(人设标签/提示词/作业策略)以 agent_id(稳定逻辑标识)同步下发至 MC 持存，由 MC 的 agent-runtime 子模块运行；承担提示词与人设管理、提示词自动生成、记忆管理、智能体构建、智能体评测；不直接操作设备。提示词工程与评测以 coze-loop(Go)旁挂集成，其余组件用 Java(智能体域特例 CON-14)。</x:v>
       </x:c>
       <x:c r="F2" s="2" t="s">
         <x:v>208</x:v>
@@ -8151,8 +8151,8 @@
       <x:c r="G2" s="3" t="s">
         <x:v>714</x:v>
       </x:c>
-      <x:c r="H2" s="3" t="s">
-        <x:v>715</x:v>
+      <x:c r="H2" s="3" t="str">
+        <x:v>R-SWM-001(提示词与人设管理)含人设标签、提示词模板库两个异构关注点(元数据/文本资产)，故拆 2 模块；运行时(场景适配/动态调用/调IRS)移至 MC 的 agent-runtime 子模块(M-MC-06)，不在 SWM；提示词自动生成(R-SWM-005)独立成 M-SWM-07；智能体定义组装与提示词包同步归构建模块(M-SWM-05)，迭代优化决策归评测模块(M-SWM-06)。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:8" ht="54">
@@ -8368,25 +8368,25 @@
         <x:v>211</x:v>
       </x:c>
       <x:c r="B11" s="4" t="s">
-        <x:v>135</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="C11" s="5" t="s">
-        <x:v>136</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="D11" s="5" t="s">
-        <x:v>137</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="E11" s="5" t="s">
-        <x:v>138</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="F11" s="5" t="s">
-        <x:v>748</x:v>
+        <x:v>760</x:v>
       </x:c>
       <x:c r="G11" s="5" t="s">
-        <x:v>749</x:v>
+        <x:v>761</x:v>
       </x:c>
       <x:c r="H11" s="5" t="s">
-        <x:v>750</x:v>
+        <x:v>762</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:8" ht="27">
@@ -8394,22 +8394,22 @@
         <x:v>215</x:v>
       </x:c>
       <x:c r="B12" s="6" t="s">
-        <x:v>751</x:v>
+        <x:v>763</x:v>
       </x:c>
       <x:c r="C12" s="7" t="s">
-        <x:v>752</x:v>
+        <x:v>764</x:v>
       </x:c>
       <x:c r="D12" s="7" t="s">
-        <x:v>721</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="E12" s="7" t="s">
-        <x:v>753</x:v>
+        <x:v>765</x:v>
       </x:c>
       <x:c r="F12" s="7" t="s">
-        <x:v>754</x:v>
+        <x:v>766</x:v>
       </x:c>
       <x:c r="G12" s="7" t="s">
-        <x:v>724</x:v>
+        <x:v>761</x:v>
       </x:c>
       <x:c r="H12" s="7" t="s">
         <x:v>220</x:v>
@@ -8420,51 +8420,51 @@
         <x:v>215</x:v>
       </x:c>
       <x:c r="B13" s="6" t="s">
-        <x:v>755</x:v>
+        <x:v>767</x:v>
       </x:c>
       <x:c r="C13" s="7" t="s">
-        <x:v>756</x:v>
+        <x:v>768</x:v>
       </x:c>
       <x:c r="D13" s="7" t="s">
-        <x:v>721</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="E13" s="7" t="s">
-        <x:v>757</x:v>
+        <x:v>769</x:v>
       </x:c>
       <x:c r="F13" s="7" t="s">
-        <x:v>758</x:v>
+        <x:v>770</x:v>
       </x:c>
       <x:c r="G13" s="7" t="s">
-        <x:v>724</x:v>
+        <x:v>761</x:v>
       </x:c>
       <x:c r="H13" s="7" t="s">
-        <x:v>759</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" spans="1:8" ht="54">
-      <x:c r="A14" s="4" t="s">
-        <x:v>211</x:v>
-      </x:c>
-      <x:c r="B14" s="4" t="s">
-        <x:v>139</x:v>
-      </x:c>
-      <x:c r="C14" s="5" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="D14" s="5" t="s">
+        <x:v>220</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:8">
+      <x:c r="A14" s="6" t="s">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="B14" s="6" t="s">
+        <x:v>771</x:v>
+      </x:c>
+      <x:c r="C14" s="7" t="s">
+        <x:v>772</x:v>
+      </x:c>
+      <x:c r="D14" s="7" t="s">
         <x:v>141</x:v>
       </x:c>
-      <x:c r="E14" s="5" t="s">
-        <x:v>142</x:v>
-      </x:c>
-      <x:c r="F14" s="5" t="s">
-        <x:v>760</x:v>
-      </x:c>
-      <x:c r="G14" s="5" t="s">
+      <x:c r="E14" s="7" t="s">
+        <x:v>773</x:v>
+      </x:c>
+      <x:c r="F14" s="7" t="s">
+        <x:v>774</x:v>
+      </x:c>
+      <x:c r="G14" s="7" t="s">
         <x:v>761</x:v>
       </x:c>
-      <x:c r="H14" s="5" t="s">
-        <x:v>762</x:v>
+      <x:c r="H14" s="7" t="s">
+        <x:v>220</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:8" ht="27">
@@ -8472,19 +8472,19 @@
         <x:v>215</x:v>
       </x:c>
       <x:c r="B15" s="6" t="s">
-        <x:v>763</x:v>
+        <x:v>775</x:v>
       </x:c>
       <x:c r="C15" s="7" t="s">
-        <x:v>764</x:v>
+        <x:v>776</x:v>
       </x:c>
       <x:c r="D15" s="7" t="s">
         <x:v>141</x:v>
       </x:c>
       <x:c r="E15" s="7" t="s">
-        <x:v>765</x:v>
+        <x:v>777</x:v>
       </x:c>
       <x:c r="F15" s="7" t="s">
-        <x:v>766</x:v>
+        <x:v>778</x:v>
       </x:c>
       <x:c r="G15" s="7" t="s">
         <x:v>761</x:v>
@@ -8493,160 +8493,160 @@
         <x:v>220</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" spans="1:8">
-      <x:c r="A16" s="6" t="s">
-        <x:v>215</x:v>
-      </x:c>
-      <x:c r="B16" s="6" t="s">
-        <x:v>767</x:v>
-      </x:c>
-      <x:c r="C16" s="7" t="s">
-        <x:v>768</x:v>
-      </x:c>
-      <x:c r="D16" s="7" t="s">
-        <x:v>141</x:v>
-      </x:c>
-      <x:c r="E16" s="7" t="s">
-        <x:v>769</x:v>
-      </x:c>
-      <x:c r="F16" s="7" t="s">
-        <x:v>770</x:v>
-      </x:c>
-      <x:c r="G16" s="7" t="s">
-        <x:v>761</x:v>
-      </x:c>
-      <x:c r="H16" s="7" t="s">
-        <x:v>220</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" spans="1:8">
+    <x:row r="16" spans="1:8" ht="81">
+      <x:c r="A16" s="4" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="B16" s="4" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="C16" s="5" t="s">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="D16" s="5" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="E16" s="5" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="F16" s="5" t="s">
+        <x:v>779</x:v>
+      </x:c>
+      <x:c r="G16" s="5" t="s">
+        <x:v>780</x:v>
+      </x:c>
+      <x:c r="H16" s="5" t="s">
+        <x:v>781</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" spans="1:8" ht="27">
       <x:c r="A17" s="6" t="s">
         <x:v>215</x:v>
       </x:c>
       <x:c r="B17" s="6" t="s">
-        <x:v>771</x:v>
+        <x:v>782</x:v>
       </x:c>
       <x:c r="C17" s="7" t="s">
-        <x:v>772</x:v>
+        <x:v>783</x:v>
       </x:c>
       <x:c r="D17" s="7" t="s">
-        <x:v>141</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="E17" s="7" t="s">
-        <x:v>773</x:v>
+        <x:v>784</x:v>
       </x:c>
       <x:c r="F17" s="7" t="s">
-        <x:v>774</x:v>
+        <x:v>785</x:v>
       </x:c>
       <x:c r="G17" s="7" t="s">
-        <x:v>761</x:v>
+        <x:v>780</x:v>
       </x:c>
       <x:c r="H17" s="7" t="s">
         <x:v>220</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" spans="1:8" ht="27">
+    <x:row r="18" spans="1:8" ht="31.5">
       <x:c r="A18" s="6" t="s">
         <x:v>215</x:v>
       </x:c>
       <x:c r="B18" s="6" t="s">
-        <x:v>775</x:v>
+        <x:v>786</x:v>
       </x:c>
       <x:c r="C18" s="7" t="s">
-        <x:v>776</x:v>
+        <x:v>787</x:v>
       </x:c>
       <x:c r="D18" s="7" t="s">
-        <x:v>141</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="E18" s="7" t="s">
-        <x:v>777</x:v>
+        <x:v>788</x:v>
       </x:c>
       <x:c r="F18" s="7" t="s">
-        <x:v>778</x:v>
+        <x:v>789</x:v>
       </x:c>
       <x:c r="G18" s="7" t="s">
-        <x:v>761</x:v>
+        <x:v>780</x:v>
       </x:c>
       <x:c r="H18" s="7" t="s">
-        <x:v>220</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" spans="1:8" ht="81">
-      <x:c r="A19" s="4" t="s">
-        <x:v>211</x:v>
-      </x:c>
-      <x:c r="B19" s="4" t="s">
-        <x:v>143</x:v>
-      </x:c>
-      <x:c r="C19" s="5" t="s">
-        <x:v>144</x:v>
-      </x:c>
-      <x:c r="D19" s="5" t="s">
+        <x:v>790</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" spans="1:8" ht="27">
+      <x:c r="A19" s="6" t="s">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="B19" s="6" t="s">
+        <x:v>791</x:v>
+      </x:c>
+      <x:c r="C19" s="7" t="s">
+        <x:v>792</x:v>
+      </x:c>
+      <x:c r="D19" s="7" t="s">
         <x:v>145</x:v>
       </x:c>
-      <x:c r="E19" s="5" t="s">
-        <x:v>146</x:v>
-      </x:c>
-      <x:c r="F19" s="5" t="s">
-        <x:v>779</x:v>
-      </x:c>
-      <x:c r="G19" s="5" t="s">
+      <x:c r="E19" s="7" t="s">
+        <x:v>793</x:v>
+      </x:c>
+      <x:c r="F19" s="7" t="s">
+        <x:v>794</x:v>
+      </x:c>
+      <x:c r="G19" s="7" t="s">
         <x:v>780</x:v>
       </x:c>
-      <x:c r="H19" s="5" t="s">
-        <x:v>781</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" spans="1:8" ht="27">
+      <x:c r="H19" s="7" t="s">
+        <x:v>584</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" spans="1:8">
       <x:c r="A20" s="6" t="s">
         <x:v>215</x:v>
       </x:c>
       <x:c r="B20" s="6" t="s">
-        <x:v>782</x:v>
+        <x:v>795</x:v>
       </x:c>
       <x:c r="C20" s="7" t="s">
-        <x:v>783</x:v>
+        <x:v>796</x:v>
       </x:c>
       <x:c r="D20" s="7" t="s">
         <x:v>145</x:v>
       </x:c>
       <x:c r="E20" s="7" t="s">
-        <x:v>784</x:v>
+        <x:v>797</x:v>
       </x:c>
       <x:c r="F20" s="7" t="s">
-        <x:v>785</x:v>
+        <x:v>798</x:v>
       </x:c>
       <x:c r="G20" s="7" t="s">
         <x:v>780</x:v>
       </x:c>
       <x:c r="H20" s="7" t="s">
-        <x:v>220</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" spans="1:8" ht="31.5">
-      <x:c r="A21" s="6" t="s">
-        <x:v>215</x:v>
-      </x:c>
-      <x:c r="B21" s="6" t="s">
-        <x:v>786</x:v>
-      </x:c>
-      <x:c r="C21" s="7" t="s">
-        <x:v>787</x:v>
-      </x:c>
-      <x:c r="D21" s="7" t="s">
-        <x:v>145</x:v>
-      </x:c>
-      <x:c r="E21" s="7" t="s">
-        <x:v>788</x:v>
-      </x:c>
-      <x:c r="F21" s="7" t="s">
-        <x:v>789</x:v>
-      </x:c>
-      <x:c r="G21" s="7" t="s">
-        <x:v>780</x:v>
-      </x:c>
-      <x:c r="H21" s="7" t="s">
-        <x:v>790</x:v>
+        <x:v>534</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" spans="1:8" ht="108">
+      <x:c r="A21" s="4" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="B21" s="4" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="C21" s="5" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="D21" s="5" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="E21" s="5" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="F21" s="5" t="s">
+        <x:v>799</x:v>
+      </x:c>
+      <x:c r="G21" s="5" t="s">
+        <x:v>800</x:v>
+      </x:c>
+      <x:c r="H21" s="5" t="s">
+        <x:v>801</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:8" ht="27">
@@ -8654,129 +8654,129 @@
         <x:v>215</x:v>
       </x:c>
       <x:c r="B22" s="6" t="s">
-        <x:v>791</x:v>
+        <x:v>802</x:v>
       </x:c>
       <x:c r="C22" s="7" t="s">
-        <x:v>792</x:v>
+        <x:v>803</x:v>
       </x:c>
       <x:c r="D22" s="7" t="s">
-        <x:v>145</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E22" s="7" t="s">
-        <x:v>793</x:v>
+        <x:v>804</x:v>
       </x:c>
       <x:c r="F22" s="7" t="s">
-        <x:v>794</x:v>
+        <x:v>805</x:v>
       </x:c>
       <x:c r="G22" s="7" t="s">
-        <x:v>780</x:v>
+        <x:v>800</x:v>
       </x:c>
       <x:c r="H22" s="7" t="s">
-        <x:v>584</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" spans="1:8">
+        <x:v>806</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" spans="1:8" ht="67.5">
       <x:c r="A23" s="6" t="s">
         <x:v>215</x:v>
       </x:c>
       <x:c r="B23" s="6" t="s">
-        <x:v>795</x:v>
+        <x:v>807</x:v>
       </x:c>
       <x:c r="C23" s="7" t="s">
-        <x:v>796</x:v>
+        <x:v>808</x:v>
       </x:c>
       <x:c r="D23" s="7" t="s">
-        <x:v>145</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E23" s="7" t="s">
-        <x:v>797</x:v>
+        <x:v>809</x:v>
       </x:c>
       <x:c r="F23" s="7" t="s">
-        <x:v>798</x:v>
+        <x:v>810</x:v>
       </x:c>
       <x:c r="G23" s="7" t="s">
-        <x:v>780</x:v>
+        <x:v>800</x:v>
       </x:c>
       <x:c r="H23" s="7" t="s">
-        <x:v>534</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" spans="1:8" ht="108">
-      <x:c r="A24" s="4" t="s">
-        <x:v>211</x:v>
-      </x:c>
-      <x:c r="B24" s="4" t="s">
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="C24" s="5" t="s">
-        <x:v>148</x:v>
-      </x:c>
-      <x:c r="D24" s="5" t="s">
+        <x:v>811</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" spans="1:8" ht="54">
+      <x:c r="A24" s="6" t="s">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="B24" s="6" t="s">
+        <x:v>812</x:v>
+      </x:c>
+      <x:c r="C24" s="7" t="s">
+        <x:v>813</x:v>
+      </x:c>
+      <x:c r="D24" s="7" t="s">
         <x:v>149</x:v>
       </x:c>
-      <x:c r="E24" s="5" t="s">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="F24" s="5" t="s">
-        <x:v>799</x:v>
-      </x:c>
-      <x:c r="G24" s="5" t="s">
+      <x:c r="E24" s="7" t="s">
+        <x:v>814</x:v>
+      </x:c>
+      <x:c r="F24" s="7" t="s">
+        <x:v>815</x:v>
+      </x:c>
+      <x:c r="G24" s="7" t="s">
         <x:v>800</x:v>
       </x:c>
-      <x:c r="H24" s="5" t="s">
-        <x:v>801</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" spans="1:8" ht="27">
+      <x:c r="H24" s="7" t="s">
+        <x:v>816</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" spans="1:8" ht="40.5">
       <x:c r="A25" s="6" t="s">
         <x:v>215</x:v>
       </x:c>
       <x:c r="B25" s="6" t="s">
-        <x:v>802</x:v>
+        <x:v>817</x:v>
       </x:c>
       <x:c r="C25" s="7" t="s">
-        <x:v>803</x:v>
+        <x:v>818</x:v>
       </x:c>
       <x:c r="D25" s="7" t="s">
         <x:v>149</x:v>
       </x:c>
       <x:c r="E25" s="7" t="s">
-        <x:v>804</x:v>
+        <x:v>819</x:v>
       </x:c>
       <x:c r="F25" s="7" t="s">
-        <x:v>805</x:v>
+        <x:v>820</x:v>
       </x:c>
       <x:c r="G25" s="7" t="s">
         <x:v>800</x:v>
       </x:c>
       <x:c r="H25" s="7" t="s">
-        <x:v>806</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" spans="1:8" ht="67.5">
+        <x:v>220</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" spans="1:8" ht="40.5">
       <x:c r="A26" s="6" t="s">
         <x:v>215</x:v>
       </x:c>
       <x:c r="B26" s="6" t="s">
-        <x:v>807</x:v>
+        <x:v>821</x:v>
       </x:c>
       <x:c r="C26" s="7" t="s">
-        <x:v>808</x:v>
+        <x:v>822</x:v>
       </x:c>
       <x:c r="D26" s="7" t="s">
         <x:v>149</x:v>
       </x:c>
       <x:c r="E26" s="7" t="s">
-        <x:v>809</x:v>
+        <x:v>823</x:v>
       </x:c>
       <x:c r="F26" s="7" t="s">
-        <x:v>810</x:v>
+        <x:v>824</x:v>
       </x:c>
       <x:c r="G26" s="7" t="s">
         <x:v>800</x:v>
       </x:c>
       <x:c r="H26" s="7" t="s">
-        <x:v>811</x:v>
+        <x:v>825</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:8" ht="54">
@@ -8784,103 +8784,74 @@
         <x:v>215</x:v>
       </x:c>
       <x:c r="B27" s="6" t="s">
-        <x:v>812</x:v>
+        <x:v>826</x:v>
       </x:c>
       <x:c r="C27" s="7" t="s">
-        <x:v>813</x:v>
+        <x:v>827</x:v>
       </x:c>
       <x:c r="D27" s="7" t="s">
         <x:v>149</x:v>
       </x:c>
       <x:c r="E27" s="7" t="s">
-        <x:v>814</x:v>
+        <x:v>828</x:v>
       </x:c>
       <x:c r="F27" s="7" t="s">
-        <x:v>815</x:v>
+        <x:v>829</x:v>
       </x:c>
       <x:c r="G27" s="7" t="s">
         <x:v>800</x:v>
       </x:c>
       <x:c r="H27" s="7" t="s">
-        <x:v>816</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" spans="1:8" ht="40.5">
-      <x:c r="A28" s="6" t="s">
-        <x:v>215</x:v>
-      </x:c>
-      <x:c r="B28" s="6" t="s">
-        <x:v>817</x:v>
-      </x:c>
-      <x:c r="C28" s="7" t="s">
-        <x:v>818</x:v>
-      </x:c>
-      <x:c r="D28" s="7" t="s">
+        <x:v>220</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="B28" t="str">
+        <x:v>M-SWM-07</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>按账号与画像自动生成提示词（提示词自动生成引擎）</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>R-SWM-005</x:v>
+      </x:c>
+      <x:c r="E28" t="str">
+        <x:v>根据账号主数据(MC)与用户画像(OCC 全维度档案)经 IRS 本地大模型自动生成贴合人设的提示词，降低人工编写成本；生成结果版本化并可作为智能体构建(M-SWM-05)的提示词来源。</x:v>
+      </x:c>
+      <x:c r="F28" t="str">
+        <x:v>F-SWM-07-01 账号与画像拉取；F-SWM-07-02 提示词自动生成；F-SWM-07-03 生成结果版本化与纳入构建</x:v>
+      </x:c>
+      <x:c r="G28" t="str">
+        <x:v>SRS R-SWM-005</x:v>
+      </x:c>
+      <x:c r="H28" t="str">
+        <x:v>对应 R-SWM-005。07-01 从 MC 拉账号(II-01)、从 OCC 拉画像(II-18/R-OCC-004)；07-02 经 IRS(EI-05)生成；07-03 版本化回写提示词库并可纳入构建。生成推理不经执行网关(CON-10)、私有化(CON-06)。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" spans="1:8" ht="108">
+      <x:c r="A28" s="4" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="B28" s="4" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="C28" s="5" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="D28" s="5" t="s">
         <x:v>149</x:v>
       </x:c>
-      <x:c r="E28" s="7" t="s">
-        <x:v>819</x:v>
-      </x:c>
-      <x:c r="F28" s="7" t="s">
-        <x:v>820</x:v>
-      </x:c>
-      <x:c r="G28" s="7" t="s">
+      <x:c r="E28" s="5" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="F28" s="5" t="s">
+        <x:v>799</x:v>
+      </x:c>
+      <x:c r="G28" s="5" t="s">
         <x:v>800</x:v>
       </x:c>
-      <x:c r="H28" s="7" t="s">
-        <x:v>220</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" spans="1:8" ht="40.5">
-      <x:c r="A29" s="6" t="s">
-        <x:v>215</x:v>
-      </x:c>
-      <x:c r="B29" s="6" t="s">
-        <x:v>821</x:v>
-      </x:c>
-      <x:c r="C29" s="7" t="s">
-        <x:v>822</x:v>
-      </x:c>
-      <x:c r="D29" s="7" t="s">
-        <x:v>149</x:v>
-      </x:c>
-      <x:c r="E29" s="7" t="s">
-        <x:v>823</x:v>
-      </x:c>
-      <x:c r="F29" s="7" t="s">
-        <x:v>824</x:v>
-      </x:c>
-      <x:c r="G29" s="7" t="s">
-        <x:v>800</x:v>
-      </x:c>
-      <x:c r="H29" s="7" t="s">
-        <x:v>825</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" spans="1:8" ht="54">
-      <x:c r="A30" s="6" t="s">
-        <x:v>215</x:v>
-      </x:c>
-      <x:c r="B30" s="6" t="s">
-        <x:v>826</x:v>
-      </x:c>
-      <x:c r="C30" s="7" t="s">
-        <x:v>827</x:v>
-      </x:c>
-      <x:c r="D30" s="7" t="s">
-        <x:v>149</x:v>
-      </x:c>
-      <x:c r="E30" s="7" t="s">
-        <x:v>828</x:v>
-      </x:c>
-      <x:c r="F30" s="7" t="s">
-        <x:v>829</x:v>
-      </x:c>
-      <x:c r="G30" s="7" t="s">
-        <x:v>800</x:v>
-      </x:c>
-      <x:c r="H30" s="7" t="s">
-        <x:v>220</x:v>
+      <x:c r="H28" s="5" t="s">
+        <x:v>801</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-07-14 17:35:34
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/软件概要设计-模块功能拆分-v2.xlsx
+++ b/公司项目/认知作战/文档/软件概要设计-模块功能拆分-v2.xlsx
@@ -4582,8 +4582,8 @@
       <x:c r="C30" t="s">
         <x:v>124</x:v>
       </x:c>
-      <x:c r="F30" t="s">
-        <x:v>125</x:v>
+      <x:c r="F30" t="str">
+        <x:v>R-SWM-001~005</x:v>
       </x:c>
       <x:c r="G30" s="8" t="s">
         <x:v>126</x:v>
@@ -4619,55 +4619,55 @@
     </x:row>
     <x:row r="33" spans="1:7" ht="36">
       <x:c r="D33" t="s">
-        <x:v>135</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="E33" t="s">
-        <x:v>136</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="F33" t="s">
-        <x:v>137</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="G33" s="8" t="s">
-        <x:v>138</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" spans="1:7" ht="36">
+        <x:v>142</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" spans="1:7" ht="54">
       <x:c r="D34" t="s">
-        <x:v>139</x:v>
-      </x:c>
-      <x:c r="E34" t="s">
-        <x:v>140</x:v>
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="E34" t="str">
+        <x:v>智能体构建与提示词包下发（智能体装配工厂）</x:v>
       </x:c>
       <x:c r="F34" t="s">
-        <x:v>141</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="G34" s="8" t="s">
-        <x:v>142</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" spans="1:7" ht="54">
+        <x:v>146</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" spans="1:7" ht="72">
       <x:c r="D35" t="s">
-        <x:v>143</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="E35" t="s">
-        <x:v>144</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="F35" t="s">
-        <x:v>145</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="G35" s="8" t="s">
-        <x:v>146</x:v>
+        <x:v>150</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="1:7" ht="72">
-      <x:c r="D36" t="s">
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="E36" t="s">
-        <x:v>148</x:v>
-      </x:c>
-      <x:c r="F36" t="s">
-        <x:v>149</x:v>
+      <x:c r="D36" t="str">
+        <x:v>M-SWM-07</x:v>
+      </x:c>
+      <x:c r="E36" t="str">
+        <x:v>按账号与画像自动生成提示词（提示词自动生成引擎）</x:v>
+      </x:c>
+      <x:c r="F36" t="str">
+        <x:v>R-SWM-005</x:v>
       </x:c>
       <x:c r="G36" s="8" t="s">
         <x:v>150</x:v>
@@ -6152,17 +6152,17 @@
       <x:c r="D30" s="7" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="E30" s="7" t="s">
-        <x:v>421</x:v>
-      </x:c>
-      <x:c r="F30" s="7" t="s">
-        <x:v>422</x:v>
+      <x:c r="E30" s="7" t="str">
+        <x:v>由 MC 的 agent-runtime 子模块按 MC 持存的提示词包运行(场景适配/动态调用/读记忆/调 IRS 视觉推理与规划)自主决策动作；agent-runtime 与执行网关逻辑隔离，推理不经网关，产出的动作指令再经网关落地。</x:v>
+      </x:c>
+      <x:c r="F30" s="7" t="str">
+        <x:v>agent-runtime 运行提示词包；读记忆(R-SWM-002)；调 IRS 推理；动作经网关落地</x:v>
       </x:c>
       <x:c r="G30" s="7" t="s">
         <x:v>423</x:v>
       </x:c>
-      <x:c r="H30" s="7" t="s">
-        <x:v>424</x:v>
+      <x:c r="H30" s="7" t="str">
+        <x:v>对接 EI-05/II-08；agent-runtime 承接原 SWM M-SWM-03 运行时职责</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:8" ht="40.5">
@@ -8500,23 +8500,23 @@
       <x:c r="B16" s="4" t="s">
         <x:v>143</x:v>
       </x:c>
-      <x:c r="C16" s="5" t="s">
-        <x:v>144</x:v>
+      <x:c r="C16" s="5" t="str">
+        <x:v>智能体构建与提示词包下发（智能体装配工厂）</x:v>
       </x:c>
       <x:c r="D16" s="5" t="s">
         <x:v>145</x:v>
       </x:c>
-      <x:c r="E16" s="5" t="s">
-        <x:v>146</x:v>
-      </x:c>
-      <x:c r="F16" s="5" t="s">
-        <x:v>779</x:v>
+      <x:c r="E16" s="5" t="str">
+        <x:v>根据人设标签配置提示词与作业策略，组装为提示词包(人设标签/提示词/作业策略)并以 agent_id(稳定逻辑标识)为标识，经 II-14 同步至 MC 持存、供 OCC 作战编排引用。记忆不在提示词包内，由记忆服务独立承载。</x:v>
+      </x:c>
+      <x:c r="F16" s="5" t="str">
+        <x:v>F-SWM-05-01 提示词包构建；F-SWM-05-02 账号绑定引用；F-SWM-05-03 同步至 MC 持存；F-SWM-05-04 OCC 智能体节点定义来源</x:v>
       </x:c>
       <x:c r="G16" s="5" t="s">
         <x:v>780</x:v>
       </x:c>
-      <x:c r="H16" s="5" t="s">
-        <x:v>781</x:v>
+      <x:c r="H16" s="5" t="str">
+        <x:v>对应 R-SWM-003，构建是装配链(配置策略+组装提示词包+下发)，内聚不拆；运行时(场景适配/动态调用/调IRS)移至 MC，不在 SWM。</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:8" ht="27">
@@ -8526,17 +8526,17 @@
       <x:c r="B17" s="6" t="s">
         <x:v>782</x:v>
       </x:c>
-      <x:c r="C17" s="7" t="s">
-        <x:v>783</x:v>
+      <x:c r="C17" s="7" t="str">
+        <x:v>提示词包构建</x:v>
       </x:c>
       <x:c r="D17" s="7" t="s">
         <x:v>145</x:v>
       </x:c>
-      <x:c r="E17" s="7" t="s">
-        <x:v>784</x:v>
-      </x:c>
-      <x:c r="F17" s="7" t="s">
-        <x:v>785</x:v>
+      <x:c r="E17" s="7" t="str">
+        <x:v>按人设标签配置提示词与作业策略(目标/场景/边界)，组装为提示词包，以全局唯一 agent_id(稳定逻辑标识)为标识；提示词可手动编写或由 M-SWM-07 自动生成。</x:v>
+      </x:c>
+      <x:c r="F17" s="7" t="str">
+        <x:v>人设+提示词+作业策略组装；agent_id 标识；版本子属性</x:v>
       </x:c>
       <x:c r="G17" s="7" t="s">
         <x:v>780</x:v>
@@ -8558,8 +8558,8 @@
       <x:c r="D18" s="7" t="s">
         <x:v>145</x:v>
       </x:c>
-      <x:c r="E18" s="7" t="s">
-        <x:v>788</x:v>
+      <x:c r="E18" s="7" t="str">
+        <x:v>提示词包与账号严格 1:1 绑定(agent_id↔account_id)，绑定关系由 MC 维护，本子系统构建时引用 account_id。</x:v>
       </x:c>
       <x:c r="F18" s="7" t="s">
         <x:v>789</x:v>
@@ -8584,8 +8584,8 @@
       <x:c r="D19" s="7" t="s">
         <x:v>145</x:v>
       </x:c>
-      <x:c r="E19" s="7" t="s">
-        <x:v>793</x:v>
+      <x:c r="E19" s="7" t="str">
+        <x:v>构建完成的提示词包经 II-14 同步至 MC 持存，取得持存版本号；提示词更新时以同一 agent_id 重新同步并升级版本号。</x:v>
       </x:c>
       <x:c r="F19" s="7" t="s">
         <x:v>794</x:v>
@@ -8604,14 +8604,14 @@
       <x:c r="B20" s="6" t="s">
         <x:v>795</x:v>
       </x:c>
-      <x:c r="C20" s="7" t="s">
-        <x:v>796</x:v>
+      <x:c r="C20" s="7" t="str">
+        <x:v>OCC 智能体节点定义来源</x:v>
       </x:c>
       <x:c r="D20" s="7" t="s">
         <x:v>145</x:v>
       </x:c>
-      <x:c r="E20" s="7" t="s">
-        <x:v>797</x:v>
+      <x:c r="E20" s="7" t="str">
+        <x:v>构建出的提示词包是 OCC 作战编排中智能体节点的定义来源。</x:v>
       </x:c>
       <x:c r="F20" s="7" t="s">
         <x:v>798</x:v>
@@ -8828,6 +8828,66 @@
         <x:v>对应 R-SWM-005。07-01 从 MC 拉账号(II-01)、从 OCC 拉画像(II-18/R-OCC-004)；07-02 经 IRS(EI-05)生成；07-03 版本化回写提示词库并可纳入构建。生成推理不经执行网关(CON-10)、私有化(CON-06)。</x:v>
       </x:c>
     </x:row>
+    <x:row r="29">
+      <x:c r="B29" t="str">
+        <x:v>F-SWM-07-01</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>账号与画像拉取</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>R-SWM-005</x:v>
+      </x:c>
+      <x:c r="E29" t="str">
+        <x:v>按 account_id 从 MC 拉取账号主数据(II-01)，按目标标识从 OCC 拉取用户画像(II-18，来源于 R-OCC-004 全维度档案)。</x:v>
+      </x:c>
+      <x:c r="F29" t="str">
+        <x:v>账号主数据拉取；用户画像拉取；只引用标识不复制主数据</x:v>
+      </x:c>
+      <x:c r="G29" t="str">
+        <x:v>SRS R-SWM-005</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="B30" t="str">
+        <x:v>F-SWM-07-02</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>提示词自动生成</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>R-SWM-005</x:v>
+      </x:c>
+      <x:c r="E30" t="str">
+        <x:v>将账号属性与用户画像作为上下文，经 IRS 本地大模型推理(EI-05，不经执行网关)生成贴合人设的提示词。</x:v>
+      </x:c>
+      <x:c r="F30" t="str">
+        <x:v>上下文组装；IRS 生成推理；私有化约束</x:v>
+      </x:c>
+      <x:c r="G30" t="str">
+        <x:v>SRS R-SWM-005</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="B31" t="str">
+        <x:v>F-SWM-07-03</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>生成结果版本化与纳入构建</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>R-SWM-005</x:v>
+      </x:c>
+      <x:c r="E31" t="str">
+        <x:v>生成的提示词纳入版本管理(以 agent_id 索引)，回写提示词库，可由工程师审核微调后纳入 R-SWM-003 智能体构建。</x:v>
+      </x:c>
+      <x:c r="F31" t="str">
+        <x:v>版本化回写；人工审核微调；纳入构建</x:v>
+      </x:c>
+      <x:c r="G31" t="str">
+        <x:v>SRS R-SWM-005</x:v>
+      </x:c>
+    </x:row>
     <x:row r="28" spans="1:8" ht="108">
       <x:c r="A28" s="4" t="s">
         <x:v>211</x:v>
@@ -8852,6 +8912,84 @@
       </x:c>
       <x:c r="H28" s="5" t="s">
         <x:v>801</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" spans="1:8" ht="27">
+      <x:c r="A29" s="6" t="s">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="B29" s="6" t="s">
+        <x:v>802</x:v>
+      </x:c>
+      <x:c r="C29" s="7" t="s">
+        <x:v>803</x:v>
+      </x:c>
+      <x:c r="D29" s="7" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="E29" s="7" t="s">
+        <x:v>804</x:v>
+      </x:c>
+      <x:c r="F29" s="7" t="s">
+        <x:v>805</x:v>
+      </x:c>
+      <x:c r="G29" s="7" t="s">
+        <x:v>800</x:v>
+      </x:c>
+      <x:c r="H29" s="7" t="s">
+        <x:v>806</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" spans="1:8" ht="27">
+      <x:c r="A30" s="6" t="s">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="B30" s="6" t="s">
+        <x:v>802</x:v>
+      </x:c>
+      <x:c r="C30" s="7" t="s">
+        <x:v>803</x:v>
+      </x:c>
+      <x:c r="D30" s="7" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="E30" s="7" t="s">
+        <x:v>804</x:v>
+      </x:c>
+      <x:c r="F30" s="7" t="s">
+        <x:v>805</x:v>
+      </x:c>
+      <x:c r="G30" s="7" t="s">
+        <x:v>800</x:v>
+      </x:c>
+      <x:c r="H30" s="7" t="s">
+        <x:v>806</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" spans="1:8" ht="27">
+      <x:c r="A31" s="6" t="s">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="B31" s="6" t="s">
+        <x:v>802</x:v>
+      </x:c>
+      <x:c r="C31" s="7" t="s">
+        <x:v>803</x:v>
+      </x:c>
+      <x:c r="D31" s="7" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="E31" s="7" t="s">
+        <x:v>804</x:v>
+      </x:c>
+      <x:c r="F31" s="7" t="s">
+        <x:v>805</x:v>
+      </x:c>
+      <x:c r="G31" s="7" t="s">
+        <x:v>800</x:v>
+      </x:c>
+      <x:c r="H31" s="7" t="s">
+        <x:v>806</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-07-17 13:59:44
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/软件概要设计-模块功能拆分-v2.xlsx
+++ b/公司项目/认知作战/文档/软件概要设计-模块功能拆分-v2.xlsx
@@ -4380,8 +4380,8 @@
       <x:c r="F16" t="s">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="G16" s="8" t="s">
-        <x:v>68</x:v>
+      <x:c r="G16" s="8" t="str">
+        <x:v>承载养号、账号-终端-代理绑定、登录状态维护等可自动化的账号操作的执行编排，以及养号拟人化节奏策略（内置）。认知行动账号经移动端 ADB/无障碍通道养号、爬虫账号经桌面端 CDP 通道养护。</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:7" ht="72">
@@ -4408,8 +4408,8 @@
       <x:c r="F18" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="G18" s="8" t="s">
-        <x:v>76</x:v>
+      <x:c r="G18" s="8" t="str">
+        <x:v>平台级权威源，唯一维护社交媒体账号主数据（注册、凭据、验证、风险评估、生命周期、账号分类），经事件总线向 DC/SWM/OCC 分发 account_id，保证全网一致、凭据加密、被封账号全网即时失效；账号分爬虫账号(桌面端)与认知行动账号(移动端)两类。</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:7" ht="54">
@@ -4430,14 +4430,14 @@
       <x:c r="D20" t="s">
         <x:v>81</x:v>
       </x:c>
-      <x:c r="E20" t="s">
-        <x:v>82</x:v>
+      <x:c r="E20" t="str">
+        <x:v>智能体账号绑定与资产迁移（四元行动单元）</x:v>
       </x:c>
       <x:c r="F20" t="s">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="G20" s="8" t="s">
-        <x:v>84</x:v>
+      <x:c r="G20" s="8" t="str">
+        <x:v>维护账号与智能体定义（agent_id）严格 1:1 绑定，叠加账号-终端-代理绑定形成四元行动单元（agent_id:account_id:终端:代理 IP = 1:1:1:1）；账号被封后支持资产迁移整体继承人格（提示词版本/记忆）。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:7" ht="90">
@@ -4450,8 +4450,8 @@
       <x:c r="F21" t="s">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="G21" s="8" t="s">
-        <x:v>88</x:v>
+      <x:c r="G21" s="8" t="str">
+        <x:v>作为智能体执行宿主，接收并持存 SWM 同步来的智能体定义（以 agent_id 为标识，含提示词/作业策略），任务执行时调用这些定义驱动设备作业，执行前校验行为风格一致性（不一致拒绝执行）；确立「SWM 定义中心、MC 执行宿主」分工。</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:7" ht="36">
@@ -4585,22 +4585,22 @@
       <x:c r="F30" t="str">
         <x:v>R-SWM-001~005</x:v>
       </x:c>
-      <x:c r="G30" s="8" t="s">
-        <x:v>126</x:v>
+      <x:c r="G30" s="8" t="str">
+        <x:v>执行层的「智能体定义与记忆中心」：编写驱动智能体作业的提示词与记忆，将提示词包(提示词/作业策略)以 agent_id 同步下发至 MC 持存；承担智能体构建、评测、提示词管理、记忆管理；不直接操作设备。</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:7" ht="54">
       <x:c r="D31" t="s">
         <x:v>127</x:v>
       </x:c>
-      <x:c r="E31" t="s">
-        <x:v>128</x:v>
-      </x:c>
-      <x:c r="F31" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="G31" s="8" t="s">
-        <x:v>130</x:v>
+      <x:c r="E31" t="str">
+        <x:v>提示词管理（V3.9：原人设标签管理废除）</x:v>
+      </x:c>
+      <x:c r="F31" t="str">
+        <x:v>R-SWM-001(提示词)</x:v>
+      </x:c>
+      <x:c r="G31" s="8" t="str">
+        <x:v>V3.9 废除人设标签实体，改为提示词模板与版本管理（人设属性直接写进提示词文本）。</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:7" ht="54">
@@ -4627,8 +4627,8 @@
       <x:c r="F33" t="s">
         <x:v>141</x:v>
       </x:c>
-      <x:c r="G33" s="8" t="s">
-        <x:v>142</x:v>
+      <x:c r="G33" s="8" t="str">
+        <x:v>实现智能体作业记忆的存储、场景沉淀、历史复用与个性化状态延续，使智能体长期行为符合行为风格且不断演进。</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:7" ht="54">
@@ -4641,8 +4641,8 @@
       <x:c r="F34" t="s">
         <x:v>145</x:v>
       </x:c>
-      <x:c r="G34" s="8" t="s">
-        <x:v>146</x:v>
+      <x:c r="G34" s="8" t="str">
+        <x:v>编写提示词与记忆初值、配置作业策略，组装为完整智能体定义并以 agent_id 为标识，经 II-14 同步至 MC 持存、供 OCC 行动编排引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:7" ht="72">
@@ -4717,8 +4717,8 @@
       <x:c r="F39" t="s">
         <x:v>162</x:v>
       </x:c>
-      <x:c r="G39" s="8" t="s">
-        <x:v>163</x:v>
+      <x:c r="G39" s="8" t="str">
+        <x:v>全链路指挥大脑：构建「目标识别→数据分析与情报→行动编排→效果评估」行动闭环，并承担内容资源统一管理(唯一权威源)；基于 DC 采集的原始舆情/传播数据（经 II-13）与 IRS 推理产出行动方案，在本子系统内完成数据分析与情报研判（V3.3 起由 DC 移入），以行动编排直接编排 MC 中智能体节点与自动化脚本节点形成执行流程落地。</x:v>
       </x:c>
     </x:row>
     <x:row r="40" spans="1:7" ht="54">
@@ -4767,8 +4767,8 @@
       <x:c r="D43" t="s">
         <x:v>176</x:v>
       </x:c>
-      <x:c r="E43" t="s">
-        <x:v>177</x:v>
+      <x:c r="E43" t="str">
+        <x:v>行动方案规划（行动参谋）</x:v>
       </x:c>
       <x:c r="F43" t="s">
         <x:v>178</x:v>
@@ -4795,8 +4795,8 @@
       <x:c r="D45" t="s">
         <x:v>184</x:v>
       </x:c>
-      <x:c r="E45" t="s">
-        <x:v>185</x:v>
+      <x:c r="E45" t="str">
+        <x:v>效果评估（行动复盘官）</x:v>
       </x:c>
       <x:c r="F45" t="s">
         <x:v>186</x:v>
@@ -4815,8 +4815,8 @@
       <x:c r="F46" t="s">
         <x:v>190</x:v>
       </x:c>
-      <x:c r="G46" s="8" t="s">
-        <x:v>191</x:v>
+      <x:c r="G46" s="8" t="str">
+        <x:v>搭建并迭代多语种/多场景/多风格舆论作业策略库，为行动提供可复用、可演进的策略资产。</x:v>
       </x:c>
     </x:row>
     <x:row r="47" spans="1:7" ht="54">

</xml_diff>

<commit_message>
vault backup: 2026-07-20 18:16:29
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/软件概要设计-模块功能拆分-v2.xlsx
+++ b/公司项目/认知作战/文档/软件概要设计-模块功能拆分-v2.xlsx
@@ -4431,13 +4431,13 @@
         <x:v>81</x:v>
       </x:c>
       <x:c r="E20" t="str">
-        <x:v>智能体账号绑定与资产迁移（四元行动单元）</x:v>
+        <x:v>智能体账号绑定与资产迁移（行动关系 1:N:1:1）</x:v>
       </x:c>
       <x:c r="F20" t="s">
         <x:v>83</x:v>
       </x:c>
       <x:c r="G20" s="8" t="str">
-        <x:v>维护账号与智能体定义（agent_id）严格 1:1 绑定，叠加账号-终端-代理绑定形成四元行动单元（agent_id:account_id:终端:代理 IP = 1:1:1:1）；账号被封后支持资产迁移整体继承人格（提示词版本/记忆）。</x:v>
+        <x:v>维护智能体定义（agent_id）与账号（account_id）1:N 绑定（一个agent绑多账号），账号级记忆/动态提示词按 account_id 1:1 归属；叠加账号-终端-代理绑定（1:1:1）形成行动关系（agent_id:account_id:终端:代理 IP = 1:N:1:1）；账号被封后支持账号资产迁移（账号级记忆/动态提示词迁移到新账号，agent 不变）。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:7" ht="90">
@@ -4451,7 +4451,7 @@
         <x:v>87</x:v>
       </x:c>
       <x:c r="G21" s="8" t="str">
-        <x:v>作为智能体执行宿主，接收并持存 SWM 同步来的智能体定义（以 agent_id 为标识，含提示词/作业策略），任务执行时调用这些定义驱动设备作业，执行前校验行为风格一致性（不一致拒绝执行）；确立「SWM 定义中心、MC 执行宿主」分工。</x:v>
+        <x:v>作为智能体执行宿主，接收并持存 SWM 同步来的提示词包（以 agent_id+account_id 组合为标识，含提示词模板/账号级动态提示词实例/作业策略），任务执行时调用这些定义驱动设备作业，执行前校验行为风格一致性（不一致拒绝执行）；确立「SWM 提示词生成与记忆中心、MC 执行宿主」分工。</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:7" ht="36">
@@ -4586,7 +4586,7 @@
         <x:v>R-SWM-001~005</x:v>
       </x:c>
       <x:c r="G30" s="8" t="str">
-        <x:v>执行层的「智能体定义与记忆中心」：编写驱动智能体作业的提示词与记忆，将提示词包(提示词/作业策略)以 agent_id 同步下发至 MC 持存；承担智能体构建、评测、提示词管理、记忆管理；不直接操作设备。</x:v>
+        <x:v>执行层的「提示词生成与记忆中心」：编写驱动智能体作业的提示词模板与记忆，将提示词包(提示词模板/账号级动态提示词实例/作业策略)以 agent_id+account_id 组合同步下发至 MC 持存；承担智能体构建、评测、提示词管理、记忆管理；不直接操作设备。</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:7" ht="54">
@@ -4613,8 +4613,8 @@
       <x:c r="F32" t="s">
         <x:v>133</x:v>
       </x:c>
-      <x:c r="G32" s="8" t="s">
-        <x:v>134</x:v>
+      <x:c r="G32" s="8" t="str">
+        <x:v>建立提示词模板库并按用途/平台/目标分类管理；对提示词模板进行版本管理，以 agent_id 为主键索引（模板共性），账号级动态提示词实例按 account_id 1:1 归属，支持版本对比/回滚/变更记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="33" spans="1:7" ht="36">
@@ -4628,7 +4628,7 @@
         <x:v>141</x:v>
       </x:c>
       <x:c r="G33" s="8" t="str">
-        <x:v>实现智能体作业记忆的存储、场景沉淀、历史复用与个性化状态延续，使智能体长期行为符合行为风格且不断演进。</x:v>
+        <x:v>实现智能体作业记忆的存储、场景沉淀、历史复用与个性化状态延续，使智能体长期行为符合行为风格且不断演进。记忆按 account_id 1:1 归属（账号级独立）。</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:7" ht="54">
@@ -4642,7 +4642,7 @@
         <x:v>145</x:v>
       </x:c>
       <x:c r="G34" s="8" t="str">
-        <x:v>编写提示词与记忆初值、配置作业策略，组装为完整智能体定义并以 agent_id 为标识，经 II-14 同步至 MC 持存、供 OCC 行动编排引用。</x:v>
+        <x:v>编写提示词模板与记忆初值、配置作业策略，组装为完整提示词包（模板+账号级动态实例）并以 agent_id+account_id 组合为标识，经 II-14 同步至 MC 持存、供 OCC 行动编排引用。</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:7" ht="72">
@@ -6153,10 +6153,10 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="E30" s="7" t="str">
-        <x:v>由 MC 的 agent-runtime 子模块按 MC 持存的提示词包运行(场景适配/动态调用/读记忆/调 IRS 视觉推理与规划)自主决策动作；agent-runtime 与执行网关逻辑隔离，推理不经网关，产出的动作指令再经网关落地。</x:v>
+        <x:v>由 MC 的 agent-runtime 子模块按 MC 持存的提示词包运行(场景适配/动态调用/按account_id读记忆/调 IRS 视觉推理与规划)自主决策动作；agent-runtime 与执行网关逻辑隔离，推理不经网关，产出的动作指令再经网关落地。</x:v>
       </x:c>
       <x:c r="F30" s="7" t="str">
-        <x:v>agent-runtime 运行提示词包；读记忆(R-SWM-002)；调 IRS 推理；动作经网关落地</x:v>
+        <x:v>agent-runtime 运行提示词包；按account_id读记忆(R-SWM-002)；调 IRS 推理；动作经网关落地</x:v>
       </x:c>
       <x:c r="G30" s="7" t="s">
         <x:v>423</x:v>
@@ -7134,17 +7134,17 @@
       <x:c r="B68" s="4" t="s">
         <x:v>81</x:v>
       </x:c>
-      <x:c r="C68" s="5" t="s">
-        <x:v>82</x:v>
+      <x:c r="C68" s="5" t="str">
+        <x:v>智能体账号绑定与资产迁移（行动关系 1:N:1:1）</x:v>
       </x:c>
       <x:c r="D68" s="5" t="s">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="E68" s="5" t="s">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="F68" s="5" t="s">
-        <x:v>577</x:v>
+      <x:c r="E68" s="5" t="str">
+        <x:v>维护智能体定义（agent_id）与账号（account_id）1:N 绑定（一个agent绑多账号），账号级记忆/动态提示词按 account_id 1:1 归属；叠加账号-终端-代理绑定（1:1:1）形成行动关系（agent_id:account_id:终端:代理 IP = 1:N:1:1）；账号被封后支持账号资产迁移（账号级记忆/动态提示词迁移到新账号，agent 不变）。</x:v>
+      </x:c>
+      <x:c r="F68" s="5" t="str">
+        <x:v>F-MC-13-01 智能体-账号 1:N 绑定维护；F-MC-13-02 行动关系维护；F-MC-13-03 账号资产抽取；F-MC-13-04 迁移目标账号校验；F-MC-13-05 继承写入与绑定切换</x:v>
       </x:c>
       <x:c r="G68" s="5" t="s">
         <x:v>578</x:v>
@@ -7166,11 +7166,11 @@
       <x:c r="D69" s="7" t="s">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="E69" s="7" t="s">
-        <x:v>582</x:v>
-      </x:c>
-      <x:c r="F69" s="7" t="s">
-        <x:v>583</x:v>
+      <x:c r="E69" s="7" t="str">
+        <x:v>记录并维护 agent_id↔account_id 1:N 绑定关系（一个agent绑多账号）；账号级记忆/动态提示词按 account_id 1:1 归属；agent_id 由 SWM 分配经 II-14（agent_id+account_id 组合）同步至本子系统持存。</x:v>
+      </x:c>
+      <x:c r="F69" s="7" t="str">
+        <x:v>agent_id↔account_id 1:N；账号级记忆/动态提示词 account_id 1:1；记录维护</x:v>
       </x:c>
       <x:c r="G69" s="7" t="s">
         <x:v>578</x:v>
@@ -7186,17 +7186,17 @@
       <x:c r="B70" s="6" t="s">
         <x:v>585</x:v>
       </x:c>
-      <x:c r="C70" s="7" t="s">
-        <x:v>586</x:v>
+      <x:c r="C70" s="7" t="str">
+        <x:v>行动关系维护</x:v>
       </x:c>
       <x:c r="D70" s="7" t="s">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="E70" s="7" t="s">
-        <x:v>587</x:v>
-      </x:c>
-      <x:c r="F70" s="7" t="s">
-        <x:v>588</x:v>
+      <x:c r="E70" s="7" t="str">
+        <x:v>记录并维护 agent_id↔account_id↔终端↔代理 IP 行动关系，形成 1:N:1:1（agent:账号=1:N，账号:终端:IP=1:1:1）。</x:v>
+      </x:c>
+      <x:c r="F70" s="7" t="str">
+        <x:v>行动关系；1:N:1:1</x:v>
       </x:c>
       <x:c r="G70" s="7" t="s">
         <x:v>578</x:v>
@@ -7218,11 +7218,11 @@
       <x:c r="D71" s="7" t="s">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="E71" s="7" t="s">
-        <x:v>591</x:v>
-      </x:c>
-      <x:c r="F71" s="7" t="s">
-        <x:v>592</x:v>
+      <x:c r="E71" s="7" t="str">
+        <x:v>从被封禁账号抽取待迁移的账号级资产：账号级记忆数据、账号级动态提示词实例。</x:v>
+      </x:c>
+      <x:c r="F71" s="7" t="str">
+        <x:v>抽取账号级记忆/动态提示词实例；资产完整性校验</x:v>
       </x:c>
       <x:c r="G71" s="7" t="s">
         <x:v>578</x:v>
@@ -7296,8 +7296,8 @@
       <x:c r="D74" s="5" t="s">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="E74" s="5" t="s">
-        <x:v>88</x:v>
+      <x:c r="E74" s="5" t="str">
+        <x:v>作为智能体执行宿主，接收并持存 SWM 同步来的提示词包（以 agent_id+account_id 组合为标识，含提示词模板/账号级动态提示词实例/作业策略），任务执行时调用这些定义驱动设备作业，执行前校验行为风格一致性（不一致拒绝执行）；确立「SWM 提示词生成与记忆中心、MC 执行宿主」分工。</x:v>
       </x:c>
       <x:c r="F74" s="5" t="s">
         <x:v>601</x:v>
@@ -7322,8 +7322,8 @@
       <x:c r="D75" s="7" t="s">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="E75" s="7" t="s">
-        <x:v>606</x:v>
+      <x:c r="E75" s="7" t="str">
+        <x:v>以 agent_id+account_id 组合为主键接收 SWM 同步的提示词包(提示词模板/账号级动态提示词实例/作业策略)并持存，作为任务执行调用依据。</x:v>
       </x:c>
       <x:c r="F75" s="7" t="s">
         <x:v>607</x:v>
@@ -8143,7 +8143,7 @@
         <x:v>R-SWM-001~005</x:v>
       </x:c>
       <x:c r="E2" s="3" t="str">
-        <x:v>执行层的「提示词生成与记忆中心」：根据人设(画像/账号属性)生成驱动智能体作业的提示词并管理记忆，将生成的提示词包(人设标签/提示词/作业策略)以 agent_id(稳定逻辑标识)同步下发至 MC 持存，由 MC 的 agent-runtime 子模块运行；承担提示词与人设管理、提示词自动生成、记忆管理、智能体构建、智能体评测；不直接操作设备。提示词工程与评测以 coze-loop(Go)旁挂集成，其余组件用 Java(智能体域特例 CON-14)。</x:v>
+        <x:v>执行层的「提示词生成与记忆中心」：根据画像/账号属性生成驱动智能体作业的提示词模板并管理记忆，将生成的提示词包(提示词模板/账号级动态提示词实例/作业策略)以 agent_id+account_id 组合(模板按agent_id稳定逻辑标识、动态实例按account_id)同步下发至 MC 持存，由 MC 的 agent-runtime 子模块运行；承担提示词管理、提示词自动生成、记忆管理、智能体构建、智能体评测；不直接操作设备。提示词工程与评测以 coze-loop(Go)旁挂集成，其余组件用 Java(智能体域特例 CON-14)。</x:v>
       </x:c>
       <x:c r="F2" s="2" t="s">
         <x:v>208</x:v>
@@ -8246,8 +8246,8 @@
       <x:c r="D6" s="5" t="s">
         <x:v>133</x:v>
       </x:c>
-      <x:c r="E6" s="5" t="s">
-        <x:v>134</x:v>
+      <x:c r="E6" s="5" t="str">
+        <x:v>建立提示词模板库并按用途/平台/目标分类管理；对提示词模板进行版本管理，以 agent_id 为主键索引（模板共性），账号级动态提示词实例按 account_id 1:1 归属，支持版本对比/回滚/变更记录。</x:v>
       </x:c>
       <x:c r="F6" s="5" t="s">
         <x:v>729</x:v>
@@ -8298,8 +8298,8 @@
       <x:c r="D8" s="7" t="s">
         <x:v>721</x:v>
       </x:c>
-      <x:c r="E8" s="7" t="s">
-        <x:v>738</x:v>
+      <x:c r="E8" s="7" t="str">
+        <x:v>对提示词模板进行版本管理，以 agent_id 为主键索引（模板共性），账号级动态提示词实例按 account_id 索引（账号个性），支持版本对比、回滚与变更记录；版本回滚失败时告警。</x:v>
       </x:c>
       <x:c r="F8" s="7" t="s">
         <x:v>739</x:v>
@@ -8507,7 +8507,7 @@
         <x:v>145</x:v>
       </x:c>
       <x:c r="E16" s="5" t="str">
-        <x:v>根据人设标签配置提示词与作业策略，组装为提示词包(人设标签/提示词/作业策略)并以 agent_id(稳定逻辑标识)为标识，经 II-14 同步至 MC 持存、供 OCC 作战编排引用。记忆不在提示词包内，由记忆服务独立承载。</x:v>
+        <x:v>根据画像/账号属性配置提示词模板与作业策略，组装为提示词包(提示词模板/账号级动态提示词实例/作业策略)并以 agent_id+account_id 组合为标识(模板按agent_id稳定逻辑标识、动态实例按account_id)，经 II-14 同步至 MC 持存、供 OCC 作战编排引用。一个agent可绑N个账号，每账号独立动态实例。记忆不在提示词包内，由记忆服务(account_id主键)独立承载。</x:v>
       </x:c>
       <x:c r="F16" s="5" t="str">
         <x:v>F-SWM-05-01 提示词包构建；F-SWM-05-02 账号绑定引用；F-SWM-05-03 同步至 MC 持存；F-SWM-05-04 OCC 智能体节点定义来源</x:v>
@@ -8559,7 +8559,7 @@
         <x:v>145</x:v>
       </x:c>
       <x:c r="E18" s="7" t="str">
-        <x:v>提示词包与账号严格 1:1 绑定(agent_id↔account_id)，绑定关系由 MC 维护，本子系统构建时引用 account_id。</x:v>
+        <x:v>提示词模板与账号 1:N 绑定(agent_id↔account_id，一个agent绑多账号)，每账号独立动态提示词实例(account_id 1:1)；绑定关系由 MC 维护，本子系统构建时引用 account_id。</x:v>
       </x:c>
       <x:c r="F18" s="7" t="s">
         <x:v>789</x:v>
@@ -8979,8 +8979,8 @@
       <x:c r="D31" s="7" t="s">
         <x:v>149</x:v>
       </x:c>
-      <x:c r="E31" s="7" t="s">
-        <x:v>804</x:v>
+      <x:c r="E31" s="7" t="str">
+        <x:v>生成的提示词模板纳入版本管理(以 agent_id 索引，模板共性)，回写提示词库，账号级动态实例由 R-SWM-003 构建时基于模板结合账号属性生成；可由工程师审核微调后纳入 R-SWM-003 智能体构建。</x:v>
       </x:c>
       <x:c r="F31" s="7" t="s">
         <x:v>805</x:v>

</xml_diff>

<commit_message>
vault backup: 2026-07-21 08:56:48
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/软件概要设计-模块功能拆分-v2.xlsx
+++ b/公司项目/认知作战/文档/软件概要设计-模块功能拆分-v2.xlsx
@@ -3115,7 +3115,7 @@
     <x:numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <x:numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </x:numFmts>
-  <x:fonts count="24">
+  <x:fonts count="26">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -3293,6 +3293,21 @@
       <x:name val="宋体"/>
       <x:charset val="0"/>
       <x:scheme val="minor"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color theme="1"/>
+      <x:name val="宋体"/>
+      <x:charset xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" val="134"/>
+      <x:scheme xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" val="minor"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color theme="1"/>
+      <x:name val="宋体"/>
+      <x:charset xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" val="134"/>
+      <x:scheme xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" val="minor"/>
     </x:font>
   </x:fonts>
   <x:fills count="36">
@@ -3761,7 +3776,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="13">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3786,6 +3801,18 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="4" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="4" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyFont="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyFont="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="49">
@@ -4248,28 +4275,28 @@
       <x:c r="B7" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="C7" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="F7" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="G7" s="8" t="s">
-        <x:v>32</x:v>
+      <x:c r="C7" t="str">
+        <x:v>15个</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>R-MC-001~015</x:v>
+      </x:c>
+      <x:c r="G7" s="8" t="str">
+        <x:v>统一自动化执行引擎与多终端执行网关：统一管理移动端（真机/云手机/ARM 板卡/虚拟化真机）与桌面端（指纹浏览器 Profile）两类执行终端；收口所有终端动作（可观测/可审计/可熔断）；承担账号资源平台级权威源与智能体执行宿主两项职责；M-MC-15（V3.0 / V3.10 新增）承载真机 Agent 运行时与编排（CON-15 独立部署单元，借鉴 SonicCloudOrg）。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:7" ht="54">
       <x:c r="D8" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="E8" t="s">
-        <x:v>34</x:v>
+      <x:c r="E8" t="str">
+        <x:v>执行终端接入与台账（终端资源池管理者；V3.0 / V3.10 边界调整：Agent 接入归 M-MC-15，本模块回归纯台账持有方）</x:v>
       </x:c>
       <x:c r="F8" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="G8" s="8" t="s">
-        <x:v>36</x:v>
+      <x:c r="G8" s="8" t="str">
+        <x:v>维护四类执行终端（移动端真机/云手机/ARM 板卡/虚拟化真机、桌面端指纹浏览器 Profile）的台账数据库与状态查询——元数据 CRUD、分组标签、批量操作编排、REST 查询；订阅 M-MC-15 设备上下线事件写库；桌面端 Profile 创建（调 EI-06）仍归本模块。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:7" ht="72">
@@ -5450,8 +5477,8 @@
       <x:c r="D3" s="5" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="E3" s="5" t="s">
-        <x:v>36</x:v>
+      <x:c r="E3" s="5" t="str">
+        <x:v>维护四类执行终端（移动端真机/云手机/ARM 板卡/虚拟化真机、桌面端指纹浏览器 Profile）的台账数据库与状态查询——元数据 CRUD、分组标签、批量操作编排、REST 查询；订阅 M-MC-15 设备上下线事件写库；桌面端 Profile 创建（调 EI-06）仍归本模块。V3.0 / V3.10 边界调整：原 Agent 接入归 M-MC-15，本模块回归纯台账持有方。</x:v>
       </x:c>
       <x:c r="F3" s="5" t="s">
         <x:v>304</x:v>
@@ -5947,8 +5974,8 @@
       <x:c r="E22" s="5" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="F22" s="5" t="s">
-        <x:v>385</x:v>
+      <x:c r="F22" s="5" t="str">
+        <x:v>F-MC-05-01 动作收口与转发；F-MC-05-02 动作鉴权；F-MC-05-03 动作记录与上报；F-MC-05-04 异常熔断；F-MC-05-05 设备SDK接口与通道路由（V3.0 / V3.10 收缩为薄层，真机实现下沉 M-MC-15）</x:v>
       </x:c>
       <x:c r="G22" s="5" t="s">
         <x:v>386</x:v>
@@ -6068,23 +6095,23 @@
       <x:c r="B27" s="6" t="s">
         <x:v>407</x:v>
       </x:c>
-      <x:c r="C27" s="7" t="s">
-        <x:v>408</x:v>
+      <x:c r="C27" s="7" t="str">
+        <x:v>设备SDK接口与通道路由（V3.0 / V3.10 收缩为薄层）</x:v>
       </x:c>
       <x:c r="D27" s="7" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="E27" s="7" t="s">
-        <x:v>409</x:v>
-      </x:c>
-      <x:c r="F27" s="7" t="s">
-        <x:v>410</x:v>
+      <x:c r="E27" s="7" t="str">
+        <x:v>本模块只持 DeviceSdk 统一接口（click/input/screenshot/install/execute）+ DeviceChannelRouter 按 terminal_type 路由；真机 RealDeviceSdk 实现下沉 M-MC-15，桌面端 ProfileSdk（CDP 直连 EI-06）留 V1.2；移动端 ADB/无障碍、桌面端 CDP 对上层透明。</x:v>
+      </x:c>
+      <x:c r="F27" s="7" t="str">
+        <x:v>DeviceSdk 接口定义；DeviceChannelRouter 按 terminal_type 路由；真机实现下沉 M-MC-15；其余 4 SDK 留 V1.2</x:v>
       </x:c>
       <x:c r="G27" s="7" t="s">
         <x:v>386</x:v>
       </x:c>
-      <x:c r="H27" s="7" t="s">
-        <x:v>220</x:v>
+      <x:c r="H27" s="7" t="str">
+        <x:v>V3.0 / V3.10 接口/实现分离，真机实现归 M-MC-15，详见 SDD §5.2.1</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:8" ht="67.5">
@@ -7437,6 +7464,188 @@
       </x:c>
       <x:c r="H79" s="7" t="s">
         <x:v>534</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="100" customHeight="1">
+      <x:c r="A80" s="9" t="str">
+        <x:v>②模块</x:v>
+      </x:c>
+      <x:c r="B80" s="9" t="str">
+        <x:v>M-MC-15</x:v>
+      </x:c>
+      <x:c r="C80" s="10" t="str">
+        <x:v>真机 Agent 运行时与编排（真机落地执行单元，V3.0 / V3.10 新增，CON-15）</x:v>
+      </x:c>
+      <x:c r="D80" s="9" t="str">
+        <x:v>R-MC-015</x:v>
+      </x:c>
+      <x:c r="E80" s="10" t="str">
+        <x:v>作为所有真机动作的物理落地单元和 Agent 连接的生命周期管理者。双形态——M-MC-15.c 中心侧编排器（mc-service 同进程）持 II-02 WS endpoint，全权管 Agent 注册/心跳/占用锁/媒体面协商；作为 RealDeviceSdk 的实现方接收 M-MC-05 网关下发的动作。M-MC-15.a 设备主机侧 Agent 运行时（独立部署单元，每台插真机的主机一台 Spring Boot 进程）是 MC 体系内唯一触碰真机的进程，承载 ddmlib+uia2+scrcpy。借鉴 SonicCloudOrg（已 archived，Apache 2.0 fork 自维护）。</x:v>
+      </x:c>
+      <x:c r="F80" s="10" t="str">
+        <x:v>F-MC-15-01 Agent注册与鉴权握手；F-MC-15-02 心跳保活与在线状态判定；F-MC-15-03 设备占用锁；F-MC-15-04 ADB控制通道；F-MC-15-05 无障碍控制通道(uia2)；F-MC-15-06 远控画面源(scrcpy)</x:v>
+      </x:c>
+      <x:c r="G80" s="9" t="str">
+        <x:v>SRS R-MC-015</x:v>
+      </x:c>
+      <x:c r="H80" s="10" t="str">
+        <x:v>对应 R-MC-015，CON-15 Agent 独立部署单元；F-MC-05-05 真机实现下沉本模块；动作路径 M-MC-05→M-MC-15.c→II-02→M-MC-15.a→ADB/uia2/scrcpy；V1.2 加 iOS/热插拔/设备保护/远程升级</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="36" customHeight="1">
+      <x:c r="A81" s="11" t="str">
+        <x:v>③功能</x:v>
+      </x:c>
+      <x:c r="B81" s="11" t="str">
+        <x:v>F-MC-15-01</x:v>
+      </x:c>
+      <x:c r="C81" s="12" t="str">
+        <x:v>Agent 注册与鉴权握手</x:v>
+      </x:c>
+      <x:c r="D81" s="11" t="str">
+        <x:v>R-MC-015</x:v>
+      </x:c>
+      <x:c r="E81" s="12" t="str">
+        <x:v>Agent 启动经 II-02 WS 连中心侧编排器，agentKey 配置文件校验 + 版本/能力上报(auth 消息)；中心侧回 authResult 分配 agentId</x:v>
+      </x:c>
+      <x:c r="F81" s="12" t="str">
+        <x:v>agentKey 配置校验；版本/能力上报；agentId 分配</x:v>
+      </x:c>
+      <x:c r="G81" s="11" t="str">
+        <x:v>SRS R-MC-015</x:v>
+      </x:c>
+      <x:c r="H81" s="12" t="str">
+        <x:v>MVP 不做密钥轮换；Sonic TransportServer auth 对应</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="36" customHeight="1">
+      <x:c r="A82" s="11" t="str">
+        <x:v>③功能</x:v>
+      </x:c>
+      <x:c r="B82" s="11" t="str">
+        <x:v>F-MC-15-02</x:v>
+      </x:c>
+      <x:c r="C82" s="12" t="str">
+        <x:v>心跳保活与在线状态判定</x:v>
+      </x:c>
+      <x:c r="D82" s="11" t="str">
+        <x:v>R-MC-015</x:v>
+      </x:c>
+      <x:c r="E82" s="12" t="str">
+        <x:v>Agent 周期发 heartBeat(默认30s)，超时(默认90s)判掉线；推 terminal_offline 事件给 M-MC-01 更新台账在线状态</x:v>
+      </x:c>
+      <x:c r="F82" s="12" t="str">
+        <x:v>30s 心跳；90s 超时判离线；推事件给 M-MC-01</x:v>
+      </x:c>
+      <x:c r="G82" s="11" t="str">
+        <x:v>SRS R-MC-015</x:v>
+      </x:c>
+      <x:c r="H82" s="12" t="str">
+        <x:v>台账在线状态数据源</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="36" customHeight="1">
+      <x:c r="A83" s="11" t="str">
+        <x:v>③功能</x:v>
+      </x:c>
+      <x:c r="B83" s="11" t="str">
+        <x:v>F-MC-15-03</x:v>
+      </x:c>
+      <x:c r="C83" s="12" t="str">
+        <x:v>设备占用锁</x:v>
+      </x:c>
+      <x:c r="D83" s="11" t="str">
+        <x:v>R-MC-015</x:v>
+      </x:c>
+      <x:c r="E83" s="12" t="str">
+        <x:v>设备占用锁(occupy/release)，一台设备同时只让一个会话用(远控/自动化互斥)；内存锁(单 mc-service 副本)，不做分布式锁</x:v>
+      </x:c>
+      <x:c r="F83" s="12" t="str">
+        <x:v>occupy/release；远控/自动化互斥；内存锁</x:v>
+      </x:c>
+      <x:c r="G83" s="11" t="str">
+        <x:v>SRS R-MC-015</x:v>
+      </x:c>
+      <x:c r="H83" s="12" t="str">
+        <x:v>防远控和自动化并发打架；分布式锁留 V1.2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="36" customHeight="1">
+      <x:c r="A84" s="11" t="str">
+        <x:v>③功能</x:v>
+      </x:c>
+      <x:c r="B84" s="11" t="str">
+        <x:v>F-MC-15-04</x:v>
+      </x:c>
+      <x:c r="C84" s="12" t="str">
+        <x:v>ADB 控制通道</x:v>
+      </x:c>
+      <x:c r="D84" s="11" t="str">
+        <x:v>R-MC-015</x:v>
+      </x:c>
+      <x:c r="E84" s="12" t="str">
+        <x:v>ddmlib 实现 ADB 通道：install/uninstall/pressKey/reboot/screenshot；动作子集(不做交互式 shell 终端)；经 runAction 消息收口(与 F-MC-15-05 共享)</x:v>
+      </x:c>
+      <x:c r="F84" s="12" t="str">
+        <x:v>install/pressKey/reboot/screenshot；ddmlib 封装</x:v>
+      </x:c>
+      <x:c r="G84" s="11" t="str">
+        <x:v>SRS R-MC-015</x:v>
+      </x:c>
+      <x:c r="H84" s="12" t="str">
+        <x:v>Sonic AndroidDeviceBridgeTool 对应</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="36" customHeight="1">
+      <x:c r="A85" s="11" t="str">
+        <x:v>③功能</x:v>
+      </x:c>
+      <x:c r="B85" s="11" t="str">
+        <x:v>F-MC-15-05</x:v>
+      </x:c>
+      <x:c r="C85" s="12" t="str">
+        <x:v>无障碍控制通道(uia2)</x:v>
+      </x:c>
+      <x:c r="D85" s="11" t="str">
+        <x:v>R-MC-015</x:v>
+      </x:c>
+      <x:c r="E85" s="12" t="str">
+        <x:v>引 sonic-driver-core(Maven jar) 封装 uiautomator2-server：UI 元素 find/click/sendKeys/swipe；断言类步骤全砍；经 runAction 消息收口</x:v>
+      </x:c>
+      <x:c r="F85" s="12" t="str">
+        <x:v>find/click/sendKeys/swipe；sonic-driver-core 封装</x:v>
+      </x:c>
+      <x:c r="G85" s="11" t="str">
+        <x:v>SRS R-MC-015</x:v>
+      </x:c>
+      <x:c r="H85" s="12" t="str">
+        <x:v>依赖 archived 库 sonic-driver-core；uia2 协议本身稳定</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="48" customHeight="1">
+      <x:c r="A86" s="11" t="str">
+        <x:v>③功能</x:v>
+      </x:c>
+      <x:c r="B86" s="11" t="str">
+        <x:v>F-MC-15-06</x:v>
+      </x:c>
+      <x:c r="C86" s="12" t="str">
+        <x:v>远控画面源(scrcpy)</x:v>
+      </x:c>
+      <x:c r="D86" s="11" t="str">
+        <x:v>R-MC-015</x:v>
+      </x:c>
+      <x:c r="E86" s="12" t="str">
+        <x:v>抄 Sonic ScrcpyInputSocketThread/OutputSocketThread(Apache2.0)；启动 scrcpy server 抓 H.264 → 经 startScrcpy 推到 mc-sfu 指定端口；本功能只产画面源，WebRTC 转发由 M-MC-04 mc-sfu 承担</x:v>
+      </x:c>
+      <x:c r="F86" s="12" t="str">
+        <x:v>scrcpy 启动+H.264 推流到 mc-sfu；不经 mc-service WS 转发</x:v>
+      </x:c>
+      <x:c r="G86" s="11" t="str">
+        <x:v>SRS R-MC-015</x:v>
+      </x:c>
+      <x:c r="H86" s="12" t="str">
+        <x:v>画面源与转发分离；媒体面 Agent→mc-sfu 端口直推</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>